<commit_message>
Add mariadb connection, basic db backed login/signup api routes
</commit_message>
<xml_diff>
--- a/DNS Management System/Database_Tables.xlsx
+++ b/DNS Management System/Database_Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://learnermanipal-my.sharepoint.com/personal/abhishta_mitmpl2024_learner_manipal_edu/Documents/MPI intern/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2026\Internship\MPI-Internship-Projects\DNS Management System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="225" documentId="8_{C099D392-E7E4-4D23-84AC-DC991008466D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB4365BD-E892-4998-BEE7-4DE782091F2F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F0DFC8-80BC-4298-A56D-216655501F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="149">
   <si>
     <t>companies</t>
   </si>
@@ -297,9 +297,6 @@
     <t>Panel name (cPanel, AWS, etc.)</t>
   </si>
   <si>
-    <t>Hosting / DNS / SSL</t>
-  </si>
-  <si>
     <t>FK → vendors.vendor_id</t>
   </si>
   <si>
@@ -472,6 +469,21 @@
   </si>
   <si>
     <t>Admin / User/ Control</t>
+  </si>
+  <si>
+    <t>Hosting_flag</t>
+  </si>
+  <si>
+    <t>Boolean(Yes/No)</t>
+  </si>
+  <si>
+    <t>DNS_flag</t>
+  </si>
+  <si>
+    <t>SSL_flag</t>
+  </si>
+  <si>
+    <t>password</t>
   </si>
 </sst>
 </file>
@@ -552,7 +564,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -567,11 +579,7 @@
       <alignment horizontal="left" indent="5"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -579,7 +587,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -597,10 +605,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1448,7 +1452,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B96CBA7A-D56B-4CE5-9FC2-3A1847B4246A}">
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -1465,875 +1469,886 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="9" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.45">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="10"/>
-      <c r="E2" s="12" t="s">
+      <c r="D2" s="8"/>
+      <c r="E2" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="10"/>
-      <c r="I2" s="12" t="s">
+      <c r="H2" s="8"/>
+      <c r="I2" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="10" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D3" s="9"/>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="K3" s="11" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13" t="s">
+      <c r="B4" s="11"/>
+      <c r="C4" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13" t="s">
+      <c r="F4" s="11"/>
+      <c r="G4" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13" t="s">
+      <c r="J4" s="11"/>
+      <c r="K4" s="11" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13" t="s">
+      <c r="B5" s="11"/>
+      <c r="C5" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13" t="s">
+      <c r="F5" s="11"/>
+      <c r="G5" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13" t="s">
+      <c r="J5" s="11"/>
+      <c r="K5" s="11" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13" t="s">
+      <c r="B6" s="11"/>
+      <c r="C6" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="8"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
+      <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="8"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="8"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
+      <c r="B7" s="1"/>
+      <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="I9" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I11" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="K12" s="11"/>
+    </row>
+    <row r="13" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" s="11"/>
+      <c r="I13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="11"/>
+      <c r="I14" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="G15" s="11"/>
+      <c r="I15" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G16" s="11"/>
+      <c r="I16" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K16" s="11"/>
+    </row>
+    <row r="17" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G17" s="11"/>
+      <c r="I17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E18" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="D19" s="2"/>
+      <c r="E19" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G19" s="11"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E20" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E21" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E22" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E23" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E24" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E25" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E28" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E29" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I29" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J29" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="K29" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="J30" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="J31" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="K31" s="11"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="11" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
+      <c r="E32" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="J32" s="11"/>
+      <c r="K32" s="11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="11"/>
+      <c r="E33" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="J33" s="11"/>
+      <c r="K33" s="11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J34" s="11"/>
+      <c r="K34" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J35" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K35" s="11"/>
+    </row>
+    <row r="36" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="E36" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G36" s="11"/>
+      <c r="I36" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J36" s="11"/>
+      <c r="K36" s="11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="E37" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="G37" s="11"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="11"/>
+      <c r="C38" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="G38" s="11"/>
+    </row>
+    <row r="39" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="11"/>
+      <c r="C39" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="E39" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G39" s="11"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G40" s="11"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G41" s="11"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E42" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E43" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="F43" s="11"/>
+      <c r="G43" s="11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E44" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F44" s="11"/>
+      <c r="G44" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E45" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" s="11"/>
+      <c r="G45" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E48" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E49" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="F49" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="G49" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="12" t="s">
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F50" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G50" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="B51" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="C51" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="J10" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="K10" s="12" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="13" t="s">
+      <c r="E51" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="F51" s="11"/>
+      <c r="G51" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="J11" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="I12" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="J12" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="K12" s="13"/>
-    </row>
-    <row r="13" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="G13" s="13"/>
-      <c r="I13" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="G14" s="13"/>
-      <c r="I14" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
+      <c r="C52" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E52" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F52" s="11"/>
+      <c r="G52" s="11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B53" s="11"/>
+      <c r="C53" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="E53" s="11"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="11"/>
+    </row>
+    <row r="54" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A54" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B54" s="11"/>
+      <c r="C54" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E54" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F54" s="11"/>
+      <c r="G54" s="11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="B55" s="11"/>
+      <c r="C55" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="E55" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="F55" s="11"/>
+      <c r="G55" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="E56" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13" t="s">
+      <c r="B57" s="11"/>
+      <c r="C57" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="E15" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="G15" s="13"/>
-      <c r="I15" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="E16" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="13" t="s">
+      <c r="E57" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="F57" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="I16" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="J16" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="K16" s="13"/>
-    </row>
-    <row r="17" spans="1:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="D17" s="2"/>
-      <c r="E17" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="G17" s="13"/>
-      <c r="I17" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E18" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="G18" s="13"/>
-    </row>
-    <row r="19" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E19" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="G19" s="13"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E20" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="E21" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E22" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E23" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E24" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E25" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E28" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="I28" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="E29" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="F29" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="G29" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="I29" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="J29" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="K29" s="12" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F30" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="I30" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="J30" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="K30" s="13" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="C31" s="13"/>
-      <c r="E31" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="I31" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="J31" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="K31" s="13"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="I32" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="J32" s="13"/>
-      <c r="K32" s="13" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="I33" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="J33" s="13"/>
-      <c r="K33" s="13" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="I34" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="J34" s="13"/>
-      <c r="K34" s="13" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B35" s="13"/>
-      <c r="C35" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="E35" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="I35" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="J35" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="K35" s="13"/>
-    </row>
-    <row r="36" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="F36" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="G36" s="13"/>
-      <c r="I36" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="J36" s="13"/>
-      <c r="K36" s="13" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="A37" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="F37" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="G37" s="13"/>
-    </row>
-    <row r="38" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="E38" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="F38" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="G38" s="13"/>
-    </row>
-    <row r="39" spans="1:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="A39" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B39" s="13"/>
-      <c r="C39" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F39" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="G39" s="13"/>
-    </row>
-    <row r="40" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B40" s="13"/>
-      <c r="C40" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="E40" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F40" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="G40" s="13"/>
-    </row>
-    <row r="41" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E41" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="F41" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="G41" s="13"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E42" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E43" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E44" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="F44" s="13"/>
-      <c r="G44" s="13" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E45" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="F45" s="13"/>
-      <c r="G45" s="13" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A48" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E48" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B49" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="C49" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="E49" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="F49" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="G49" s="12" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A50" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="B50" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="C50" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="E50" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="F50" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G50" s="13" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A51" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="B51" s="13"/>
-      <c r="C51" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="E51" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="F51" s="13"/>
-      <c r="G51" s="13" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="B52" s="13"/>
-      <c r="C52" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="F52" s="13"/>
-      <c r="G52" s="13" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A53" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B53" s="13"/>
-      <c r="C53" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E53" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="F53" s="13"/>
-      <c r="G53" s="13" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A54" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B54" s="13"/>
-      <c r="C54" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="E54" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="F54" s="13"/>
-      <c r="G54" s="13" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E55" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="F55" s="13"/>
-      <c r="G55" s="13" t="s">
+      <c r="G57" s="11"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E58" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11" t="s">
         <v>141</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="E56" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="F56" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="G56" s="13"/>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E57" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="F57" s="13"/>
-      <c r="G57" s="13" t="s">
-        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2342,11 +2357,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2532,26 +2548,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6958310D-CFCA-49A7-8091-6AF34632A35B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA7149E8-A88B-4DF2-B4A6-57326802B1BB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2575,9 +2582,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA7149E8-A88B-4DF2-B4A6-57326802B1BB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6958310D-CFCA-49A7-8091-6AF34632A35B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add Hash Password feature
</commit_message>
<xml_diff>
--- a/DNS Management System/Database_Tables.xlsx
+++ b/DNS Management System/Database_Tables.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2026\Internship\MPI-Internship-Projects\DNS Management System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F0DFC8-80BC-4298-A56D-216655501F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09D60753-4192-404F-B5B6-5173DCE8873E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="154">
   <si>
     <t>companies</t>
   </si>
@@ -484,6 +485,21 @@
   </si>
   <si>
     <t>password</t>
+  </si>
+  <si>
+    <t>Domain Logs</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>domain snapshot at that tie</t>
+  </si>
+  <si>
+    <t>name is just enough at that time</t>
+  </si>
+  <si>
+    <t>updated values</t>
   </si>
 </sst>
 </file>
@@ -537,7 +553,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -560,11 +576,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -588,6 +615,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2356,16 +2386,951 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0731BB46-0C35-4881-871B-5F133F01CA83}">
+  <dimension ref="A1:K58"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="9" max="9" width="21.88671875" customWidth="1"/>
+    <col min="10" max="10" width="19.44140625" customWidth="1"/>
+    <col min="11" max="11" width="36.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.45">
+      <c r="A2" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="8"/>
+      <c r="E2" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="H2" s="8"/>
+      <c r="I2" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="K12" s="11"/>
+    </row>
+    <row r="13" spans="1:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" s="11"/>
+      <c r="I13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="11"/>
+      <c r="I14" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="G15" s="11"/>
+      <c r="I15" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G16" s="11"/>
+      <c r="I16" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K16" s="11"/>
+    </row>
+    <row r="17" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G17" s="11"/>
+      <c r="I17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E18" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="D19" s="2"/>
+      <c r="E19" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G19" s="11"/>
+    </row>
+    <row r="20" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E20" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E21" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E22" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E23" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E24" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E25" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E28" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E29" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I29" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J29" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="K29" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="J30" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="J31" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="K31" s="11"/>
+    </row>
+    <row r="32" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="J32" s="11"/>
+      <c r="K32" s="11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="11"/>
+      <c r="E33" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="J33" s="11"/>
+      <c r="K33" s="11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="J34" s="11"/>
+      <c r="K34" s="11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J35" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="K35" s="11"/>
+    </row>
+    <row r="36" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="E36" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G36" s="11"/>
+      <c r="I36" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J36" s="11"/>
+      <c r="K36" s="11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+      <c r="A37" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="E37" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="G37" s="11"/>
+    </row>
+    <row r="38" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A38" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="11"/>
+      <c r="C38" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="G38" s="11"/>
+    </row>
+    <row r="39" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+      <c r="A39" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="11"/>
+      <c r="C39" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="E39" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="G39" s="11"/>
+    </row>
+    <row r="40" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A40" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G40" s="11"/>
+    </row>
+    <row r="41" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B41" s="11"/>
+      <c r="C41" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G41" s="11"/>
+    </row>
+    <row r="42" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E42" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E43" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="F43" s="11"/>
+      <c r="G43" s="11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E44" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F44" s="11"/>
+      <c r="G44" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E45" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" s="11"/>
+      <c r="G45" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E48" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="I48" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="E49" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G49" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I49" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J49" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="K49" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F50" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="G50" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="I50" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="J50" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="K50" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E51" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="F51" s="11"/>
+      <c r="G51" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="I51" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="J51" s="11"/>
+      <c r="K51" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E52" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F52" s="11"/>
+      <c r="G52" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="I52" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="K52" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B53" s="11"/>
+      <c r="C53" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="E53" s="11"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="11"/>
+      <c r="I53" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A54" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B54" s="11"/>
+      <c r="C54" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E54" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F54" s="11"/>
+      <c r="G54" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="I54" s="13" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A55" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="B55" s="11"/>
+      <c r="C55" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="E55" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="F55" s="11"/>
+      <c r="G55" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A56" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="11"/>
+      <c r="C56" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="E56" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A57" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="11"/>
+      <c r="C57" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E57" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="F57" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G57" s="11"/>
+    </row>
+    <row r="58" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E58" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B22F92EFD500384AB56EB5E0F8001265" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="547ce5ca2743f0b047a162cac16b4076">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9c9fc778587b7c957cd3f52c639382f9" ns3:_="">
     <xsd:import namespace="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6"/>
@@ -2547,6 +3512,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2556,14 +3530,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA7149E8-A88B-4DF2-B4A6-57326802B1BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7E7B4CC-64D0-4DD7-B463-A7F283136F18}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2577,6 +3543,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA7149E8-A88B-4DF2-B4A6-57326802B1BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Change db excel file
</commit_message>
<xml_diff>
--- a/DNS Management System/Database_Tables.xlsx
+++ b/DNS Management System/Database_Tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2026\Internship\MPI-Internship-Projects\DNS Management System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09D60753-4192-404F-B5B6-5173DCE8873E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3503B125-A715-4F0B-9656-291A4D76C9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="156">
   <si>
     <t>companies</t>
   </si>
@@ -500,6 +500,12 @@
   </si>
   <si>
     <t>updated values</t>
+  </si>
+  <si>
+    <t>fk</t>
+  </si>
+  <si>
+    <t>compnaies.company_id</t>
   </si>
 </sst>
 </file>
@@ -591,7 +597,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -617,7 +623,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2519,7 +2528,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>14</v>
       </c>
@@ -2527,7 +2536,15 @@
       <c r="C6" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="E6" s="1"/>
+      <c r="E6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
@@ -2576,7 +2593,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -2722,7 +2739,7 @@
       </c>
       <c r="K16" s="11"/>
     </row>
-    <row r="17" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>14</v>
       </c>
@@ -2745,7 +2762,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E18" s="11" t="s">
         <v>22</v>
       </c>
@@ -2754,7 +2771,7 @@
       </c>
       <c r="G18" s="11"/>
     </row>
-    <row r="19" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D19" s="2"/>
       <c r="E19" s="11" t="s">
         <v>23</v>
@@ -2764,7 +2781,7 @@
       </c>
       <c r="G19" s="11"/>
     </row>
-    <row r="20" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E20" s="11" t="s">
         <v>24</v>
       </c>
@@ -2773,7 +2790,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E21" s="11" t="s">
         <v>25</v>
       </c>
@@ -2791,7 +2808,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E23" s="11" t="s">
         <v>14</v>
       </c>
@@ -2800,7 +2817,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E24" s="11" t="s">
         <v>27</v>
       </c>
@@ -2809,7 +2826,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E25" s="11" t="s">
         <v>28</v>
       </c>
@@ -2826,7 +2843,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E29" s="10" t="s">
         <v>69</v>
       </c>
@@ -2846,7 +2863,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>118</v>
       </c>
@@ -2869,7 +2886,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
         <v>69</v>
       </c>
@@ -2894,7 +2911,7 @@
       </c>
       <c r="K31" s="11"/>
     </row>
-    <row r="32" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
         <v>36</v>
       </c>
@@ -2919,7 +2936,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
         <v>18</v>
       </c>
@@ -2965,7 +2982,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
         <v>38</v>
       </c>
@@ -2988,7 +3005,7 @@
       </c>
       <c r="K35" s="11"/>
     </row>
-    <row r="36" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>39</v>
       </c>
@@ -3011,7 +3028,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
         <v>40</v>
       </c>
@@ -3043,7 +3060,7 @@
       </c>
       <c r="G38" s="11"/>
     </row>
-    <row r="39" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
         <v>42</v>
       </c>
@@ -3059,7 +3076,7 @@
       </c>
       <c r="G39" s="11"/>
     </row>
-    <row r="40" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
         <v>43</v>
       </c>
@@ -3075,7 +3092,7 @@
       </c>
       <c r="G40" s="11"/>
     </row>
-    <row r="41" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
         <v>27</v>
       </c>
@@ -3107,7 +3124,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E43" s="11" t="s">
         <v>51</v>
       </c>
@@ -3125,7 +3142,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E45" s="11" t="s">
         <v>14</v>
       </c>
@@ -3268,7 +3285,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="11" t="s">
         <v>148</v>
       </c>
@@ -3284,7 +3301,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="11" t="s">
         <v>59</v>
       </c>
@@ -3300,7 +3317,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
         <v>14</v>
       </c>
@@ -3316,7 +3333,7 @@
       </c>
       <c r="G57" s="11"/>
     </row>
-    <row r="58" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E58" s="11" t="s">
         <v>68</v>
       </c>
@@ -3331,6 +3348,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B22F92EFD500384AB56EB5E0F8001265" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="547ce5ca2743f0b047a162cac16b4076">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9c9fc778587b7c957cd3f52c639382f9" ns3:_="">
     <xsd:import namespace="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6"/>
@@ -3512,24 +3546,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6958310D-CFCA-49A7-8091-6AF34632A35B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA7149E8-A88B-4DF2-B4A6-57326802B1BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7E7B4CC-64D0-4DD7-B463-A7F283136F18}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3547,30 +3588,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA7149E8-A88B-4DF2-B4A6-57326802B1BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6958310D-CFCA-49A7-8091-6AF34632A35B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="fd3fa446-5203-48d5-95a2-7c0c8e2b0ba6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{29bebd42-f1ff-4c3d-9688-067e3460dc1f}" enabled="0" method="" siteId="{29bebd42-f1ff-4c3d-9688-067e3460dc1f}" removed="1"/>

</xml_diff>